<commit_message>
fix: reconcile photo lineage by record id
</commit_message>
<xml_diff>
--- a/Sierra_Estates_Units_With_Photos.xlsx
+++ b/Sierra_Estates_Units_With_Photos.xlsx
@@ -802,45 +802,14 @@
       </c>
       <c r="AH6" s="5" t="inlineStr">
         <is>
-          <t>IMG-20260810-WA0000.jpg
-IMG-20260810-WA0062.jpg
-IMG-20260810-WA0063.jpg
-IMG-20260810-WA0064.jpg
-IMG-20260810-WA0065.jpg
-IMG-20260810-WA0069.jpg
-IMG-20260810-WA0070.jpg
-IMG-20260810-WA0071.jpg
-IMG-20260810-WA0073.jpg
-IMG-20260810-WA0074.jpg
-IMG-20260810-WA0075.jpg
-IMG-20260810-WA0077.jpg
-IMG-20260810-WA0079.jpg
-STK-20260416-WA0018.webp
-VID-20260809-WA0001.mp4
-VID-20260811-WA0073.mp4
-VID-20260812-WA0029.mp4</t>
+          <t>IMG-20260810-WA0063.jpg
+IMG-20260810-WA0077.jpg</t>
         </is>
       </c>
       <c r="AI6" s="5" t="inlineStr">
         <is>
-          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0054_d4dbf51d.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0057_27e7575f.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0058_88cb2376.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0065_40f45f3b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0067_27d675c8.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0041_c76b2f16.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0042_0a39111b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0044_b14c192f.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0045_0168fb0e.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0046_a62b624a.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0048_5be77cc0.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0049_02818572.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0050_f7c468b8.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0051_92a9569a.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0052_3419c8c6.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0053_515c1855.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0054_6f743a61.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260416-WA0018_8a75b8f0.webp</t>
+          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0063_11205d91.jpg
+https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0077_7c870594.jpg</t>
         </is>
       </c>
     </row>
@@ -978,27 +947,13 @@
       <c r="AH7" s="5" t="inlineStr">
         <is>
           <t>IMG-20260810-WA0000.jpg
-IMG-20260810-WA0001.jpg
-IMG-20260810-WA0003.jpg
-IMG-20260810-WA0005.jpg
-IMG-20260810-WA0006.jpg
-IMG-20260810-WA0007.jpg
-IMG-20260810-WA0009.jpg
-IMG-20260810-WA0010.jpg
-IMG-20260810-WA0012.jpg
-IMG-20260810-WA0015.jpg
-IMG-20260810-WA0021.jpg
-IMG-20260810-WA0077.jpg
-STK-20260416-WA0018.webp
-VID-20260809-WA0001.mp4
-VID-20260810-WA0061.mp4
-VID-20260811-WA0073.mp4
-VID-20260812-WA0029.mp4</t>
+IMG-20260810-WA0010.jpg</t>
         </is>
       </c>
       <c r="AI7" s="5" t="inlineStr">
         <is>
-          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260812-WA0045_58fd2d65.webp</t>
+          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0000_79f262af.jpg
+https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0010_75963abb.jpg</t>
         </is>
       </c>
     </row>
@@ -1096,42 +1051,14 @@
       </c>
       <c r="AH8" s="5" t="inlineStr">
         <is>
-          <t>IMG-20260808-WA0123.jpg
-IMG-20260808-WA0125.jpg
-IMG-20260808-WA0126.jpg
-IMG-20260808-WA0128.jpg
-IMG-20260808-WA0129.jpg
-IMG-20260808-WA0130.jpg
-IMG-20260808-WA0132.jpg
-IMG-20260808-WA0133.jpg
-IMG-20260808-WA0134.jpg
-IMG-20260808-WA0135.jpg
-IMG-20260808-WA0136.jpg
-IMG-20260808-WA0138.jpg
-IMG-20260812-WA0046.jpg
-IMG-20260812-WA0047.jpg
-IMG-20260812-WA0048.jpg
-IMG-20260812-WA0050.jpg
-IMG-20260812-WA0051.jpg
-IMG-20260812-WA0059.jpg
-IMG-20260812-WA0064.jpg
-STK-20260812-WA0045.webp
-VID-20260812-WA0065.mp4</t>
+          <t>IMG-20260808-WA0126.jpg
+IMG-20260808-WA0134.jpg</t>
         </is>
       </c>
       <c r="AI8" s="5" t="inlineStr">
         <is>
-          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0068_001919c5.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0069_e2a58af6.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0071_263e9f04.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0072_bb27981b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0073_6ce1a86a.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0074_c7c3bd96.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0075_e3c1ab16.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0076_eae55d32.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0077_c8231555.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0078_7200e0f1.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260416-WA0018_8a75b8f0.webp</t>
+          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0126_ea3df351.jpg
+https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0134_e0759feb.jpg</t>
         </is>
       </c>
     </row>
@@ -1368,21 +1295,7 @@
       </c>
       <c r="AI10" s="5" t="inlineStr">
         <is>
-          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260313-WA0054_5f5ba7cd.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260313-WA0059_71ce10ee.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260313-WA0061_3dc4b52f.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260313-WA0062_f29aeb49.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0069_e2a58af6.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0070_21e9946b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0072_bb27981b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0073_6ce1a86a.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0074_c7c3bd96.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0076_eae55d32.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0077_c8231555.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0078_7200e0f1.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0079_16f94fff.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260817-WA0001_a9cf23af.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260416-WA0018_8a75b8f0.webp</t>
+          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260812-WA0045_58fd2d65.webp</t>
         </is>
       </c>
     </row>
@@ -1493,19 +1406,7 @@
       </c>
       <c r="AI11" s="5" t="inlineStr">
         <is>
-          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0000_79f262af.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0001_e6e4ee33.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0003_551d7227.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0005_7f27b626.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0006_582ade69.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0007_e207e85d.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0009_fbe71611.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0010_75963abb.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0012_a0ee69a5.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0015_0f712cfb.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0021_c14ec3e3.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0077_7c870594.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260416-WA0018_8a75b8f0.webp</t>
+          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260812-WA0045_58fd2d65.webp</t>
         </is>
       </c>
     </row>
@@ -1622,42 +1523,15 @@
       </c>
       <c r="AH12" s="5" t="inlineStr">
         <is>
-          <t>IMG-20260621-WA0054.jpg
-IMG-20260621-WA0057.jpg
-IMG-20260621-WA0058.jpg
-IMG-20260621-WA0065.jpg
-IMG-20260621-WA0067.jpg
-IMG-20260815-WA0041.jpg
-IMG-20260815-WA0042.jpg
-IMG-20260815-WA0044.jpg
-IMG-20260815-WA0045.jpg
-IMG-20260815-WA0046.jpg
-IMG-20260815-WA0048.jpg
-IMG-20260815-WA0049.jpg
-IMG-20260815-WA0050.jpg
-IMG-20260815-WA0051.jpg
-IMG-20260815-WA0052.jpg
-IMG-20260815-WA0053.jpg
+          <t>IMG-20260815-WA0052.jpg
 IMG-20260815-WA0054.jpg
 STK-20260416-WA0018.webp</t>
         </is>
       </c>
       <c r="AI12" s="5" t="inlineStr">
         <is>
-          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260313-WA0062_f29aeb49.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0068_001919c5.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0069_e2a58af6.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0070_21e9946b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0071_263e9f04.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0072_bb27981b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0073_6ce1a86a.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0074_c7c3bd96.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0075_e3c1ab16.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0076_eae55d32.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0077_c8231555.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0078_7200e0f1.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0079_16f94fff.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260817-WA0001_a9cf23af.jpg
+          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0052_3419c8c6.jpg
+https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0054_6f743a61.jpg
 https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260416-WA0018_8a75b8f0.webp</t>
         </is>
       </c>
@@ -1773,29 +1647,12 @@
       </c>
       <c r="AH13" s="5" t="inlineStr">
         <is>
-          <t>IMG-20260621-WA0052.jpg
-IMG-20260621-WA0054.jpg
-IMG-20260621-WA0055.jpg
-IMG-20260621-WA0057.jpg
-IMG-20260621-WA0058.jpg
-IMG-20260621-WA0059.jpg
-IMG-20260621-WA0060.jpg
-IMG-20260621-WA0061.jpg
-IMG-20260621-WA0063.jpg
-IMG-20260621-WA0065.jpg
-IMG-20260621-WA0067.jpg
-IMG-20260815-WA0042.jpg
-IMG-20260815-WA0044.jpg
-IMG-20260815-WA0045.jpg
-IMG-20260815-WA0051.jpg
-IMG-20260815-WA0052.jpg
-IMG-20260815-WA0054.jpg
-STK-20260416-WA0018.webp</t>
+          <t>IMG-20260621-WA0065.jpg</t>
         </is>
       </c>
       <c r="AI13" s="5" t="inlineStr">
         <is>
-          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260812-WA0045_58fd2d65.webp</t>
+          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0065_40f45f3b.jpg</t>
         </is>
       </c>
     </row>
@@ -1910,41 +1767,14 @@
       </c>
       <c r="AH14" s="5" t="inlineStr">
         <is>
-          <t>IMG-20260815-WA0080.jpg
-IMG-20260815-WA0081.jpg
-IMG-20260815-WA0082.jpg
-IMG-20260815-WA0084.jpg
-IMG-20260815-WA0085.jpg
-IMG-20260815-WA0086.jpg
-IMG-20260815-WA0087.jpg
-IMG-20260815-WA0090.jpg
-IMG-20260815-WA0091.jpg
-IMG-20260815-WA0092.jpg
-IMG-20260815-WA0093.jpg
-IMG-20260815-WA0094.jpg
-STK-20260416-WA0018.webp</t>
+          <t>IMG-20260815-WA0085.jpg
+IMG-20260815-WA0094.jpg</t>
         </is>
       </c>
       <c r="AI14" s="5" t="inlineStr">
         <is>
-          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0052_a3ce76a1.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0054_d4dbf51d.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0055_23b618c0.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0057_27e7575f.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0058_88cb2376.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0059_55670226.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0060_5abd95c4.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0061_c537c233.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0063_fedb954b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0065_40f45f3b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260621-WA0067_27d675c8.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0042_0a39111b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0044_b14c192f.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0045_0168fb0e.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0051_92a9569a.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0052_3419c8c6.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0054_6f743a61.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260416-WA0018_8a75b8f0.webp</t>
+          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0085_fb789252.jpg
+https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0094_0c075d25.jpg</t>
         </is>
       </c>
     </row>
@@ -2054,34 +1884,12 @@
       </c>
       <c r="AH15" s="5" t="inlineStr">
         <is>
-          <t>IMG-20260815-WA0068.jpg
-IMG-20260815-WA0069.jpg
-IMG-20260815-WA0071.jpg
-IMG-20260815-WA0072.jpg
-IMG-20260815-WA0073.jpg
-IMG-20260815-WA0074.jpg
-IMG-20260815-WA0075.jpg
-IMG-20260815-WA0076.jpg
-IMG-20260815-WA0077.jpg
-IMG-20260815-WA0078.jpg
-STK-20260416-WA0018.webp</t>
+          <t>STK-20260416-WA0018.webp</t>
         </is>
       </c>
       <c r="AI15" s="5" t="inlineStr">
         <is>
-          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0080_89ac2086.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0081_eff5d974.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0082_e94599fe.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0084_e9742216.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0085_fb789252.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0086_0387731d.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0087_67d9d637.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0090_2aa74a4a.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0091_df62952b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0092_f163cd16.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0093_451b3bc0.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0094_0c075d25.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260416-WA0018_8a75b8f0.webp</t>
+          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260416-WA0018_8a75b8f0.webp</t>
         </is>
       </c>
     </row>
@@ -2193,39 +2001,15 @@
       </c>
       <c r="AH16" s="5" t="inlineStr">
         <is>
-          <t>IMG-20260313-WA0062.jpg
-IMG-20260815-WA0068.jpg
-IMG-20260815-WA0069.jpg
-IMG-20260815-WA0070.jpg
-IMG-20260815-WA0071.jpg
-IMG-20260815-WA0072.jpg
-IMG-20260815-WA0073.jpg
-IMG-20260815-WA0074.jpg
-IMG-20260815-WA0075.jpg
-IMG-20260815-WA0076.jpg
-IMG-20260815-WA0077.jpg
-IMG-20260815-WA0078.jpg
+          <t>IMG-20260815-WA0070.jpg
 IMG-20260815-WA0079.jpg
-IMG-20260817-WA0001.jpg
-STK-20260416-WA0018.webp
-VID-20260815-WA0055.mp4</t>
+STK-20260416-WA0018.webp</t>
         </is>
       </c>
       <c r="AI16" s="5" t="inlineStr">
         <is>
-          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0000_79f262af.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0062_0be63805.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0063_11205d91.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0064_34642ed8.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0065_b56777f0.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0069_2da0fa8c.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0070_9760db89.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0071_8268c909.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0073_83e760a6.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0074_e9c28f92.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0075_73d7275d.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0077_7c870594.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260810-WA0079_d56efaed.jpg
+          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0070_21e9946b.jpg
+https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260815-WA0079_16f94fff.jpg
 https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260416-WA0018_8a75b8f0.webp</t>
         </is>
       </c>
@@ -2344,46 +2128,12 @@
       </c>
       <c r="AH17" s="5" t="inlineStr">
         <is>
-          <t>IMG-20260313-WA0054.jpg
-IMG-20260313-WA0059.jpg
-IMG-20260313-WA0061.jpg
-IMG-20260313-WA0062.jpg
-IMG-20260815-WA0069.jpg
-IMG-20260815-WA0070.jpg
-IMG-20260815-WA0072.jpg
-IMG-20260815-WA0073.jpg
-IMG-20260815-WA0074.jpg
-IMG-20260815-WA0076.jpg
-IMG-20260815-WA0077.jpg
-IMG-20260815-WA0078.jpg
-IMG-20260815-WA0079.jpg
-IMG-20260817-WA0001.jpg
-STK-20260416-WA0018.webp
-VID-20260815-WA0055.mp4</t>
+          <t>STK-20260416-WA0018.webp</t>
         </is>
       </c>
       <c r="AI17" s="5" t="inlineStr">
         <is>
-          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0123_9c9f674b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0125_9cde5c2b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0126_ea3df351.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0128_0ade1fc0.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0129_9bb32e24.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0130_b940b177.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0132_cfe0550b.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0133_4801aac8.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0134_e0759feb.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0135_d1eeaa52.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0136_5fc3ff10.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260808-WA0138_05492773.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260812-WA0046_3ba153ec.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260812-WA0047_2e4eeaec.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260812-WA0048_a95b340e.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260812-WA0050_0c534e0e.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260812-WA0051_bcbeed90.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260812-WA0059_9f4a5a7f.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/IMG-20260812-WA0064_df6b1865.jpg
-https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260812-WA0045_58fd2d65.webp</t>
+          <t>https://sierra-rent-gg2addxq.manus.space/manus-storage/STK-20260416-WA0018_8a75b8f0.webp</t>
         </is>
       </c>
     </row>

</xml_diff>